<commit_message>
v0.2.0: apply independent review fixes (single evidence standard, anchor fixes, references)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/toolkit/ACS-Health-Maturity-Assessment.xlsx
+++ b/toolkit/ACS-Health-Maturity-Assessment.xlsx
@@ -1824,7 +1824,7 @@
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>Microsoft Defender for Cloud Apps, typically included in Microsoft 365 E5, Enterprise Mobility + Security E5 and the Defender Suite and Purview Suite add-ons. Verify against your agreement.</t>
+          <t>Microsoft Defender for Cloud Apps, typically included in Microsoft 365 E5, Enterprise Mobility + Security E5 and the Defender Suite add-on. Verify against your agreement.</t>
         </is>
       </c>
       <c r="C16" s="15" t="inlineStr">
@@ -3556,7 +3556,7 @@
       </c>
       <c r="H25" s="15" t="inlineStr">
         <is>
-          <t>• Microsoft announced a cybersecurity program for rural hospitals in June 2024 that described nonprofit pricing (up to 75% discount) for independent critical access and rural emergency hospitals and a one-year no-cost security offer for other rural hospitals; confirm current terms and availability before planning on it.
+          <t>• Microsoft announced a cybersecurity program for rural hospitals in June 2024 that described special pricing and time-limited security offers for eligible rural hospitals; confirm with your licensing partner whether it is still available and what it includes before planning on it.
 • Hospitals that are part of a health system may be covered by the system's agreement rather than individual programs; check with the parent organization.</t>
         </is>
       </c>
@@ -3577,7 +3577,7 @@
       </c>
       <c r="L25" s="15" t="inlineStr">
         <is>
-          <t>AHA, June 10, 2024 (Microsoft rural hospital program)</t>
+          <t>Microsoft rural hospital cybersecurity program, announced June 10, 2024 (AHA program flyer, December 2024)</t>
         </is>
       </c>
       <c r="M25" s="15" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="L42" s="15" t="inlineStr">
         <is>
-          <t>NIST SP 800-218 PW.8</t>
+          <t>NIST SP 800-218 PW.8; NIST CSF 2.0 PR.PS</t>
         </is>
       </c>
       <c r="M42" s="15" t="inlineStr">
@@ -4978,7 +4978,7 @@
       </c>
       <c r="L44" s="15" t="inlineStr">
         <is>
-          <t>NIST CSF 2.0 GV.PO; NIST SP 800-218 PO.3</t>
+          <t>NIST CSF 2.0 GV.PO; NIST SP 800-218 PO.3; NIST SP 800-218A</t>
         </is>
       </c>
       <c r="M44" s="15" t="inlineStr">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="L52" s="15" t="inlineStr">
         <is>
-          <t>HIPAA 45 CFR 164.310(d)(2); NIST CSF 2.0 PR.DS</t>
+          <t>HIPAA 45 CFR 164.310(d)(2)(iv); NIST CSF 2.0 PR.DS</t>
         </is>
       </c>
       <c r="M52" s="15" t="inlineStr">
@@ -6698,7 +6698,7 @@
       </c>
       <c r="L67" s="15" t="inlineStr">
         <is>
-          <t>HIPAA 45 CFR 164.308(b); NIST CSF 2.0 GV.SC</t>
+          <t>HIPAA 45 CFR 164.308(b); HIPAA 45 CFR 164.314(a)(2)(i)(C); NIST CSF 2.0 GV.SC</t>
         </is>
       </c>
       <c r="M67" s="15" t="inlineStr">
@@ -7596,7 +7596,7 @@
       </c>
       <c r="L79" s="15" t="inlineStr">
         <is>
-          <t>NIST CSF 2.0 ID.IM</t>
+          <t>NIST CSF 2.0 ID.RA-06; NIST CSF 2.0 ID.IM</t>
         </is>
       </c>
       <c r="M79" s="15" t="inlineStr">
@@ -12900,7 +12900,7 @@
           <t>0 - Not in place – Departed staff accounts stay active and licensed until someone notices.
 1 - Initial – IT disables accounts when a manager remembers to tell them; licenses are rarely removed.
 2 - Developing – HR notifies IT of employee departures, but contractors, students, agency and vendor accounts are missed and licenses are removed weeks later or not at all.
-3 - Defined – Every departure (employee, contractor, student, agency, vendor) triggers account disablement within one business day and license removal per policy, verified by monthly reconciliation with HR and contract lists.
+3 - Defined – Every departure (employee, contractor, student, agency, vendor) triggers account disablement within one business day (or a shorter, documented timeframe) and license removal per policy, verified by monthly reconciliation with HR and contract lists.
 4 - Optimized – Disablement is automated from HR and sponsor records, the reconciliation shows no unexplained active accounts, and reharvested licenses are reused.</t>
         </is>
       </c>
@@ -13101,7 +13101,7 @@
       <c r="D18" s="15" t="inlineStr">
         <is>
           <t>0 - Not in place – Conditional Access is licensed but no policies exist; MFA is not required.
-1 - Initial – Security defaults or per-user MFA cover some administrators or volunteers only.
+1 - Initial – MFA relies on security defaults or per-user MFA, for some or all users; no Conditional Access policies exist.
 2 - Developing – Conditional Access requires MFA for most users, but clinical units, vendors or service accounts are excluded without review, or policies are in report-only mode.
 3 - Defined – Licensed Conditional Access policies enforce MFA for all users, administrators, vendors and remote access, with documented and approved exclusions and legacy authentication blocked.
 4 - Optimized – Policies include device compliance and, where licensed, risk-based conditions; phishing-resistant methods are required for administrators; coverage is reported and reviewed.</t>
@@ -13583,7 +13583,7 @@
       <c r="F25" s="15" t="inlineStr"/>
       <c r="G25" s="15" t="inlineStr">
         <is>
-          <t>AHA, June 10, 2024 (Microsoft rural hospital program)</t>
+          <t>Microsoft rural hospital cybersecurity program, announced June 10, 2024 (AHA program flyer, December 2024)</t>
         </is>
       </c>
       <c r="H25" s="16" t="n">
@@ -14846,7 +14846,7 @@
       <c r="F18" s="15" t="inlineStr"/>
       <c r="G18" s="15" t="inlineStr">
         <is>
-          <t>NIST SP 800-218 PW.8</t>
+          <t>NIST SP 800-218 PW.8; NIST CSF 2.0 PR.PS</t>
         </is>
       </c>
       <c r="H18" s="16" t="n">
@@ -14976,7 +14976,7 @@
       <c r="F20" s="15" t="inlineStr"/>
       <c r="G20" s="15" t="inlineStr">
         <is>
-          <t>NIST CSF 2.0 GV.PO; NIST SP 800-218 PO.3</t>
+          <t>NIST CSF 2.0 GV.PO; NIST SP 800-218 PO.3; NIST SP 800-218A</t>
         </is>
       </c>
       <c r="H20" s="16" t="n">
@@ -15500,7 +15500,7 @@
       <c r="F28" s="15" t="inlineStr"/>
       <c r="G28" s="15" t="inlineStr">
         <is>
-          <t>HIPAA 45 CFR 164.310(d)(2); NIST CSF 2.0 PR.DS</t>
+          <t>HIPAA 45 CFR 164.310(d)(2)(iv); NIST CSF 2.0 PR.DS</t>
         </is>
       </c>
       <c r="H28" s="16" t="n">
@@ -15671,7 +15671,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="171" customHeight="1">
+    <row r="5" ht="184" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
           <t>ZT-01</t>
@@ -15692,7 +15692,7 @@
           <t>0 - Not in place – No MFA, or MFA only for a few volunteers.
 1 - Initial – MFA on some remote access (for example the VPN) but not on email or administrator accounts.
 2 - Developing – MFA on remote access and email for most users; exceptions are undocumented; administrators use SMS or voice; vendor accounts are excluded.
-3 - Defined – MFA is enforced (not report-only) for all remote access, email, administrators and third-party/vendor access; exceptions are documented, approved and reviewed.
+3 - Defined – MFA is enforced (not report-only) for all remote access, email, administrators and third-party/vendor access; administrators do not use SMS or voice; exceptions are documented, approved and reviewed.
 4 - Optimized – Phishing-resistant methods (FIDO2 security keys, Windows Hello for Business or certificate-based authentication) are required for administrators and remote access; legacy authentication is blocked; coverage is monitored and gaps raise alerts.</t>
         </is>
       </c>
@@ -15900,7 +15900,7 @@
           <t>0 - Not in place – Accounts are disabled only when someone remembers; former staff and vendors remain active.
 1 - Initial – HR emails IT about departures and IT disables directory accounts, but application, remote access and vendor accounts are missed.
 2 - Developing – A documented offboarding checklist covers the directory and main applications, but timing varies, contractors and vendors are not always included and nobody reconciles.
-3 - Defined – Access for employees, contractors, students, volunteers and vendors is revoked within a defined timeframe (for example 24 hours) across directory, EHR and remote access, verified by monthly reconciliation.
+3 - Defined – Access for employees, contractors, students, volunteers and vendors is revoked within one business day (or a shorter, documented timeframe) across directory, EHR and remote access, verified by monthly reconciliation.
 4 - Optimized – Revocation is triggered automatically from HR and vendor-contract records, covers connected applications, and reconciliation exceptions are tracked to closure.</t>
         </is>
       </c>
@@ -16669,7 +16669,7 @@
       </c>
       <c r="G19" s="15" t="inlineStr">
         <is>
-          <t>HIPAA 45 CFR 164.308(b); NIST CSF 2.0 GV.SC</t>
+          <t>HIPAA 45 CFR 164.308(b); HIPAA 45 CFR 164.314(a)(2)(i)(C); NIST CSF 2.0 GV.SC</t>
         </is>
       </c>
       <c r="H19" s="16" t="n">
@@ -17477,7 +17477,7 @@
       </c>
       <c r="G31" s="15" t="inlineStr">
         <is>
-          <t>NIST CSF 2.0 ID.IM</t>
+          <t>NIST CSF 2.0 ID.RA-06; NIST CSF 2.0 ID.IM</t>
         </is>
       </c>
       <c r="H31" s="16" t="n">

</xml_diff>